<commit_message>
changement dans neutre et debut anglais
</commit_message>
<xml_diff>
--- a/Data_communes/lib_familles_produits.xlsx
+++ b/Data_communes/lib_familles_produits.xlsx
@@ -2031,10 +2031,10 @@
     <t>EAUX MINERALES, BOISSONS RAFRAICHISSANTES, JUS DE FRUITS ET DE LEGUMES</t>
   </si>
   <si>
-    <t>Eaux minerales, boissons rafraichissantes, jus de fruits et de légumes</t>
-  </si>
-  <si>
     <t>de l'</t>
+  </si>
+  <si>
+    <t>Eaux minérales, boissons rafraîchissantes, jus de fruits et de légumes</t>
   </si>
 </sst>
 </file>
@@ -2826,7 +2826,7 @@
         <v>667</v>
       </c>
       <c r="E18" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>249</v>
@@ -2981,7 +2981,7 @@
         <v>33</v>
       </c>
       <c r="C25" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>34</v>
@@ -5189,7 +5189,7 @@
         <v>163</v>
       </c>
       <c r="C121" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>164</v>

</xml_diff>